<commit_message>
freeze all players when one disconnects (Pause for countdown)
</commit_message>
<xml_diff>
--- a/Disconnect.xlsx
+++ b/Disconnect.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_NewDudo\Dudo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7883ABE7-4DF3-412B-AE7E-C31E6E290148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DED7FC3-CD8C-4310-A832-FCADDEFB584B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
   <si>
     <t>no countdown</t>
   </si>
@@ -49,13 +49,22 @@
   </si>
   <si>
     <t>Game in progress: NO</t>
+  </si>
+  <si>
+    <t>restart round</t>
+  </si>
+  <si>
+    <t>bidding</t>
+  </si>
+  <si>
+    <t>doubt in progress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -66,6 +75,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -91,9 +106,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -374,21 +390,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B4:E11"/>
+  <dimension ref="B4:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="4.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" customWidth="1"/>
     <col min="4" max="4" width="17.42578125" customWidth="1"/>
     <col min="5" max="5" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
@@ -399,7 +415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="s">
         <v>3</v>
       </c>
@@ -410,12 +426,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
@@ -426,7 +442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
         <v>2</v>
       </c>
@@ -437,12 +453,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>3</v>
       </c>
       <c r="D11" t="s">
         <v>4</v>
+      </c>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>